<commit_message>
feat: implement AI underwriting workflow, including LangGraph nodes, document parsers, extractors, and frontend dashboard components
</commit_message>
<xml_diff>
--- a/docs/applications/APP-001/income_details.xlsx
+++ b/docs/applications/APP-001/income_details.xlsx
@@ -28,13 +28,13 @@
     <t xml:space="preserve">Applicant</t>
   </si>
   <si>
-    <t xml:space="preserve">Rahul Mehta</t>
+    <t xml:space="preserve">Arjun Nair</t>
   </si>
   <si>
     <t xml:space="preserve">Applicant ID</t>
   </si>
   <si>
-    <t xml:space="preserve">APP-001</t>
+    <t xml:space="preserve">APP-003</t>
   </si>
   <si>
     <t xml:space="preserve">Employment type</t>
@@ -522,7 +522,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -550,20 +550,20 @@
         <v>16</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>60000</v>
+        <v>75000</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>30000</v>
+        <v>37500</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>42000</v>
+        <v>52500</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">B10+C10+D10-E10</f>
-        <v>120000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -571,20 +571,20 @@
         <v>17</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>60000</v>
+        <v>75000</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>30000</v>
+        <v>37500</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>42000</v>
+        <v>52500</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">B11+C11+D11-E11</f>
-        <v>120000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -592,20 +592,20 @@
         <v>18</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>60000</v>
+        <v>75000</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>30000</v>
+        <v>37500</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>42000</v>
+        <v>52500</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">B12+C12+D12-E12</f>
-        <v>120000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -614,7 +614,7 @@
       </c>
       <c r="F13" s="6" t="n">
         <f aca="false">AVERAGE(F10:F12)</f>
-        <v>120000</v>
+        <v>150000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>